<commit_message>
revision of project description
</commit_message>
<xml_diff>
--- a/Projects/lea-immenkamp/data.xlsx
+++ b/Projects/lea-immenkamp/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unitc-my.sharepoint.com/personal/zxojr58_s-cloud_uni-tuebingen_de/Documents/Module/SoSe26/Github Data project/Projects/lea-immenkamp/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0EC5C667-73CB-E445-9EC3-73BDE6A8773C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{0EC5C667-73CB-E445-9EC3-73BDE6A8773C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2ED6C578-2459-1741-90A1-9A99873CA643}"/>
   <bookViews>
     <workbookView xWindow="5180" yWindow="740" windowWidth="16700" windowHeight="16740" activeTab="1" xr2:uid="{70FB358B-DD8C-0B42-867B-04313AA7864A}"/>
   </bookViews>
@@ -81,9 +81,6 @@
     <t>id child</t>
   </si>
   <si>
-    <t>id age?</t>
-  </si>
-  <si>
     <t>i1t0</t>
   </si>
   <si>
@@ -97,6 +94,9 @@
   </si>
   <si>
     <t>sweet4</t>
+  </si>
+  <si>
+    <t>id age</t>
   </si>
 </sst>
 </file>
@@ -500,7 +500,7 @@
         <v>11</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>7</v>
@@ -6189,19 +6189,19 @@
         <v>13</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>18</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">

</xml_diff>